<commit_message>
chore: actualizar plantilla de entrada 5W1H
Por que:
- Habia cambios locales pendientes en la plantilla y se solicitó subirlos para mantener el repositorio alineado con el entorno de trabajo actual.

Que cambio:
- Se actualizo el archivo Plantilla_Entrada_5W1H.xlsx.

Impacto:
- El repositorio conserva la version mas reciente de la plantilla usada en ejecuciones actuales.

Trade-offs o riesgos:
- Al ser un archivo binario, no se puede auditar diff de contenido en git; cualquier ajuste posterior requerira validacion manual en Excel.
</commit_message>
<xml_diff>
--- a/Plantilla_Entrada_5W1H.xlsx
+++ b/Plantilla_Entrada_5W1H.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\NavaG\Downloads\5W1H\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1067D103-CA82-46B7-9A9B-3721CEA694B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5F27897-3C90-41A2-B47B-07A874DFCBBA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-105" yWindow="0" windowWidth="26010" windowHeight="20985" tabRatio="949" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>

</xml_diff>

<commit_message>
feat: actualizar plantilla con ejemplo de datos del cliente
Por que:
- Se necesitaba que la plantilla mostrara de forma explicita un ejemplo con datos del cliente para guiar el llenado correcto.

Que cambio:
- Se actualizo Plantilla_Entrada_5W1H.xlsx incorporando la estructura de ejemplo con datos del cliente.
- Se mantiene el flujo de entrada existente, pero con una referencia mas clara para usuarios nuevos.

Impacto:
- Reduce errores de captura y acelera el inicio de uso al tener una muestra concreta dentro de la plantilla.
- Mejora la consistencia de los archivos de entrada que luego se procesan en el generador.

Trade-offs o riesgos:
- Al incluir ejemplos dentro de la plantilla, se requiere cuidado para no confundir datos de ejemplo con datos finales.
- Cualquier cambio futuro en el formato de entrada obliga a mantener este ejemplo sincronizado.
</commit_message>
<xml_diff>
--- a/Plantilla_Entrada_5W1H.xlsx
+++ b/Plantilla_Entrada_5W1H.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\NavaG\Downloads\5W1H\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5F27897-3C90-41A2-B47B-07A874DFCBBA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FFF2708A-2556-49B9-92AC-195BD74E60F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="26010" windowHeight="20985" tabRatio="949" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="26010" windowHeight="20985" tabRatio="949" firstSheet="3" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="1" r:id="rId1"/>
@@ -1017,7 +1017,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="401" uniqueCount="281">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="408" uniqueCount="284">
   <si>
     <t>Plantilla de Entrada 5W1H</t>
   </si>
@@ -1860,13 +1860,22 @@
   </si>
   <si>
     <t>U/L/K/T/R/M/H</t>
+  </si>
+  <si>
+    <t>Ventas_3</t>
+  </si>
+  <si>
+    <t>Ventas_2</t>
+  </si>
+  <si>
+    <t>Ventas_0</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1914,6 +1923,12 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="11">
@@ -1994,7 +2009,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -2035,6 +2050,7 @@
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="6" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2056,13 +2072,13 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>15</xdr:col>
+      <xdr:col>16</xdr:col>
       <xdr:colOff>595842</xdr:colOff>
       <xdr:row>0</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>23</xdr:col>
+      <xdr:col>24</xdr:col>
       <xdr:colOff>9526</xdr:colOff>
       <xdr:row>20</xdr:row>
       <xdr:rowOff>3734</xdr:rowOff>
@@ -2100,13 +2116,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>8</xdr:col>
+      <xdr:col>9</xdr:col>
       <xdr:colOff>295276</xdr:colOff>
       <xdr:row>0</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>15</xdr:col>
+      <xdr:col>16</xdr:col>
       <xdr:colOff>470960</xdr:colOff>
       <xdr:row>13</xdr:row>
       <xdr:rowOff>106164</xdr:rowOff>
@@ -3712,39 +3728,42 @@
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{85A3A67E-8AC6-4000-96DE-0ABA21917A59}">
-  <dimension ref="A1:G174"/>
+  <dimension ref="A1:H174"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>98</v>
       </c>
-      <c r="B1" t="s">
-        <v>68</v>
-      </c>
-      <c r="C1" t="s">
-        <v>84</v>
-      </c>
-      <c r="D1" s="19"/>
-      <c r="E1" t="s">
+      <c r="E1" s="19"/>
+      <c r="F1" t="s">
         <v>98</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>99</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>101</v>
       </c>
-      <c r="E2" t="s">
+      <c r="B2" t="s">
+        <v>68</v>
+      </c>
+      <c r="C2" t="s">
+        <v>84</v>
+      </c>
+      <c r="D2" t="s">
+        <v>283</v>
+      </c>
+      <c r="F2" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>102</v>
       </c>
@@ -3754,17 +3773,20 @@
       <c r="C3">
         <v>973</v>
       </c>
-      <c r="E3" t="s">
+      <c r="D3" s="22">
+        <v>1831275</v>
+      </c>
+      <c r="F3" t="s">
         <v>103</v>
       </c>
-      <c r="F3">
+      <c r="G3">
         <v>10944760</v>
       </c>
-      <c r="G3">
+      <c r="H3">
         <v>10923380</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>104</v>
       </c>
@@ -3774,17 +3796,20 @@
       <c r="C4">
         <v>961</v>
       </c>
-      <c r="E4" t="s">
+      <c r="D4" s="22">
+        <v>1831275</v>
+      </c>
+      <c r="F4" t="s">
         <v>105</v>
-      </c>
-      <c r="F4">
-        <v>100</v>
       </c>
       <c r="G4">
         <v>100</v>
       </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H4">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>106</v>
       </c>
@@ -3794,17 +3819,20 @@
       <c r="C5">
         <v>998</v>
       </c>
-      <c r="E5" t="s">
+      <c r="D5" s="22">
+        <v>1831275</v>
+      </c>
+      <c r="F5" t="s">
         <v>107</v>
       </c>
-      <c r="F5">
+      <c r="G5">
         <v>10945</v>
       </c>
-      <c r="G5">
+      <c r="H5">
         <v>10923</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>108</v>
       </c>
@@ -3814,17 +3842,20 @@
       <c r="C6">
         <v>988</v>
       </c>
-      <c r="E6" t="s">
+      <c r="D6" s="22">
+        <v>1831275</v>
+      </c>
+      <c r="F6" t="s">
         <v>109</v>
       </c>
-      <c r="F6">
+      <c r="G6">
         <v>48240360</v>
       </c>
-      <c r="G6">
+      <c r="H6">
         <v>47738220</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>110</v>
       </c>
@@ -3834,17 +3865,20 @@
       <c r="C7">
         <v>1042</v>
       </c>
-      <c r="E7" t="s">
+      <c r="D7" s="22">
+        <v>1831275</v>
+      </c>
+      <c r="F7" t="s">
         <v>111</v>
-      </c>
-      <c r="F7">
-        <v>100</v>
       </c>
       <c r="G7">
         <v>100</v>
       </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H7">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>112</v>
       </c>
@@ -3854,17 +3888,20 @@
       <c r="C8">
         <v>958</v>
       </c>
-      <c r="E8" t="s">
+      <c r="D8" s="22">
+        <v>1831275</v>
+      </c>
+      <c r="F8" t="s">
         <v>113</v>
       </c>
-      <c r="F8">
+      <c r="G8">
         <v>48240360</v>
       </c>
-      <c r="G8">
+      <c r="H8">
         <v>47738220</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>114</v>
       </c>
@@ -3874,17 +3911,20 @@
       <c r="C9">
         <v>957</v>
       </c>
-      <c r="E9" t="s">
+      <c r="D9" s="22">
+        <v>1831275</v>
+      </c>
+      <c r="F9" t="s">
         <v>115</v>
-      </c>
-      <c r="F9">
-        <v>100</v>
       </c>
       <c r="G9">
         <v>100</v>
       </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H9">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>116</v>
       </c>
@@ -3894,17 +3934,20 @@
       <c r="C10">
         <v>921</v>
       </c>
-      <c r="E10" t="s">
+      <c r="D10" s="22">
+        <v>1831275</v>
+      </c>
+      <c r="F10" t="s">
         <v>117</v>
       </c>
-      <c r="F10">
+      <c r="G10">
         <v>86.3</v>
       </c>
-      <c r="G10">
+      <c r="H10">
         <v>89.3</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>118</v>
       </c>
@@ -3914,17 +3957,20 @@
       <c r="C11">
         <v>846</v>
       </c>
-      <c r="E11" t="s">
+      <c r="D11" s="22">
+        <v>1831275</v>
+      </c>
+      <c r="F11" t="s">
         <v>119</v>
-      </c>
-      <c r="F11">
-        <v>100</v>
       </c>
       <c r="G11">
         <v>100</v>
       </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H11">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>120</v>
       </c>
@@ -3934,17 +3980,20 @@
       <c r="C12">
         <v>926</v>
       </c>
-      <c r="E12" t="s">
+      <c r="D12" s="22">
+        <v>1831275</v>
+      </c>
+      <c r="F12" t="s">
         <v>121</v>
       </c>
-      <c r="F12">
+      <c r="G12">
         <v>3.64</v>
       </c>
-      <c r="G12">
+      <c r="H12">
         <v>3.42</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>122</v>
       </c>
@@ -3954,17 +4003,20 @@
       <c r="C13">
         <v>858</v>
       </c>
-      <c r="E13" t="s">
+      <c r="D13" s="22">
+        <v>1831275</v>
+      </c>
+      <c r="F13" t="s">
         <v>123</v>
       </c>
-      <c r="F13">
+      <c r="G13">
         <v>16.059999999999999</v>
       </c>
-      <c r="G13">
+      <c r="H13">
         <v>14.95</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>124</v>
       </c>
@@ -3974,17 +4026,20 @@
       <c r="C14">
         <v>941</v>
       </c>
-      <c r="E14" t="s">
+      <c r="D14" s="22">
+        <v>1831275</v>
+      </c>
+      <c r="F14" t="s">
         <v>125</v>
       </c>
-      <c r="F14">
+      <c r="G14">
         <v>16.059999999999999</v>
       </c>
-      <c r="G14">
+      <c r="H14">
         <v>14.95</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>126</v>
       </c>
@@ -3994,17 +4049,20 @@
       <c r="C15">
         <v>923</v>
       </c>
-      <c r="E15" t="s">
+      <c r="D15" s="22">
+        <v>1831274</v>
+      </c>
+      <c r="F15" t="s">
         <v>127</v>
       </c>
-      <c r="F15">
+      <c r="G15">
         <v>0.5</v>
       </c>
-      <c r="G15">
+      <c r="H15">
         <v>0.52</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>128</v>
       </c>
@@ -4014,17 +4072,20 @@
       <c r="C16">
         <v>891</v>
       </c>
-      <c r="E16" t="s">
+      <c r="D16" s="22">
+        <v>1831274</v>
+      </c>
+      <c r="F16" t="s">
         <v>129</v>
       </c>
-      <c r="F16">
+      <c r="G16">
         <v>2.2000000000000002</v>
       </c>
-      <c r="G16">
+      <c r="H16">
         <v>2.2799999999999998</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>130</v>
       </c>
@@ -4034,17 +4095,20 @@
       <c r="C17">
         <v>958</v>
       </c>
-      <c r="E17" t="s">
+      <c r="D17" s="22">
+        <v>1831274</v>
+      </c>
+      <c r="F17" t="s">
         <v>131</v>
       </c>
-      <c r="F17">
+      <c r="G17">
         <v>2.2000000000000002</v>
       </c>
-      <c r="G17">
+      <c r="H17">
         <v>2.2799999999999998</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>132</v>
       </c>
@@ -4054,17 +4118,20 @@
       <c r="C18">
         <v>856</v>
       </c>
-      <c r="E18" t="s">
+      <c r="D18" s="22">
+        <v>1831274</v>
+      </c>
+      <c r="F18" t="s">
         <v>133</v>
       </c>
-      <c r="F18">
+      <c r="G18">
         <v>7.3</v>
       </c>
-      <c r="G18">
+      <c r="H18">
         <v>6.6</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>134</v>
       </c>
@@ -4074,17 +4141,20 @@
       <c r="C19">
         <v>865</v>
       </c>
-      <c r="E19" t="s">
+      <c r="D19" s="22">
+        <v>1831274</v>
+      </c>
+      <c r="F19" t="s">
         <v>135</v>
-      </c>
-      <c r="F19">
-        <v>4.7300000000000004</v>
       </c>
       <c r="G19">
         <v>4.7300000000000004</v>
       </c>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H19">
+        <v>4.7300000000000004</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>136</v>
       </c>
@@ -4094,17 +4164,20 @@
       <c r="C20">
         <v>814</v>
       </c>
-      <c r="E20" t="s">
+      <c r="D20" s="22">
+        <v>1831274</v>
+      </c>
+      <c r="F20" t="s">
         <v>137</v>
-      </c>
-      <c r="F20">
-        <v>4.7300000000000004</v>
       </c>
       <c r="G20">
         <v>4.7300000000000004</v>
       </c>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H20">
+        <v>4.7300000000000004</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>138</v>
       </c>
@@ -4114,17 +4187,20 @@
       <c r="C21">
         <v>809</v>
       </c>
-      <c r="E21" t="s">
+      <c r="D21" s="22">
+        <v>1831274</v>
+      </c>
+      <c r="F21" t="s">
         <v>139</v>
       </c>
-      <c r="F21">
+      <c r="G21">
         <v>3483019</v>
       </c>
-      <c r="G21">
+      <c r="H21">
         <v>3576470</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>140</v>
       </c>
@@ -4134,17 +4210,20 @@
       <c r="C22">
         <v>774</v>
       </c>
-      <c r="E22" t="s">
+      <c r="D22" s="22">
+        <v>1831274</v>
+      </c>
+      <c r="F22" t="s">
         <v>141</v>
-      </c>
-      <c r="F22">
-        <v>100</v>
       </c>
       <c r="G22">
         <v>100</v>
       </c>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H22">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>142</v>
       </c>
@@ -4154,17 +4233,20 @@
       <c r="C23">
         <v>746</v>
       </c>
-      <c r="E23" t="s">
+      <c r="D23" s="22">
+        <v>1827697</v>
+      </c>
+      <c r="F23" t="s">
         <v>143</v>
       </c>
-      <c r="F23">
+      <c r="G23">
         <v>3004475</v>
       </c>
-      <c r="G23">
+      <c r="H23">
         <v>3192965</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>144</v>
       </c>
@@ -4174,17 +4256,20 @@
       <c r="C24">
         <v>766</v>
       </c>
-      <c r="E24" t="s">
+      <c r="D24" s="22">
+        <v>1827697</v>
+      </c>
+      <c r="F24" t="s">
         <v>145</v>
-      </c>
-      <c r="F24">
-        <v>100</v>
       </c>
       <c r="G24">
         <v>100</v>
       </c>
-    </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H24">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>146</v>
       </c>
@@ -4194,17 +4279,20 @@
       <c r="C25">
         <v>753</v>
       </c>
-      <c r="E25" t="s">
+      <c r="D25" s="22">
+        <v>1827697</v>
+      </c>
+      <c r="F25" t="s">
         <v>147</v>
       </c>
-      <c r="F25">
+      <c r="G25">
         <v>4704</v>
       </c>
-      <c r="G25">
+      <c r="H25">
         <v>3728</v>
       </c>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>148</v>
       </c>
@@ -4214,17 +4302,20 @@
       <c r="C26">
         <v>743</v>
       </c>
-      <c r="E26" t="s">
+      <c r="D26" s="22">
+        <v>1827697</v>
+      </c>
+      <c r="F26" t="s">
         <v>149</v>
       </c>
-      <c r="F26">
+      <c r="G26">
         <v>3253</v>
       </c>
-      <c r="G26">
+      <c r="H26">
         <v>3026</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>150</v>
       </c>
@@ -4234,8 +4325,11 @@
       <c r="C27">
         <v>677</v>
       </c>
-    </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="D27" s="22">
+        <v>1827697</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>151</v>
       </c>
@@ -4245,11 +4339,14 @@
       <c r="C28">
         <v>689</v>
       </c>
-      <c r="E28" t="s">
+      <c r="D28" s="22">
+        <v>1827697</v>
+      </c>
+      <c r="F28" t="s">
         <v>152</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>153</v>
       </c>
@@ -4259,17 +4356,20 @@
       <c r="C29">
         <v>715</v>
       </c>
-      <c r="E29" t="s">
+      <c r="D29" s="22">
+        <v>1827697</v>
+      </c>
+      <c r="F29" t="s">
         <v>154</v>
       </c>
-      <c r="F29">
+      <c r="G29">
         <v>591438</v>
       </c>
-      <c r="G29">
+      <c r="H29">
         <v>550419</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>155</v>
       </c>
@@ -4279,17 +4379,20 @@
       <c r="C30">
         <v>673</v>
       </c>
-      <c r="E30" t="s">
+      <c r="D30" s="22">
+        <v>1827697</v>
+      </c>
+      <c r="F30" t="s">
         <v>156</v>
       </c>
-      <c r="F30">
+      <c r="G30">
         <v>5.4</v>
       </c>
-      <c r="G30">
+      <c r="H30">
         <v>5</v>
       </c>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>157</v>
       </c>
@@ -4299,17 +4402,20 @@
       <c r="C31">
         <v>719</v>
       </c>
-      <c r="E31" t="s">
+      <c r="D31" s="22">
+        <v>1827697</v>
+      </c>
+      <c r="F31" t="s">
         <v>158</v>
       </c>
-      <c r="F31">
+      <c r="G31">
         <v>591</v>
       </c>
-      <c r="G31">
+      <c r="H31">
         <v>550</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>159</v>
       </c>
@@ -4319,17 +4425,20 @@
       <c r="C32">
         <v>665</v>
       </c>
-      <c r="E32" t="s">
+      <c r="D32" s="22">
+        <v>1827697</v>
+      </c>
+      <c r="F32" t="s">
         <v>160</v>
       </c>
-      <c r="F32">
+      <c r="G32">
         <v>5927047</v>
       </c>
-      <c r="G32">
+      <c r="H32">
         <v>5826820</v>
       </c>
     </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>161</v>
       </c>
@@ -4339,17 +4448,20 @@
       <c r="C33">
         <v>1014</v>
       </c>
-      <c r="E33" t="s">
+      <c r="D33" s="22">
+        <v>1827697</v>
+      </c>
+      <c r="F33" t="s">
         <v>162</v>
       </c>
-      <c r="F33">
+      <c r="G33">
         <v>12.3</v>
       </c>
-      <c r="G33">
+      <c r="H33">
         <v>12.2</v>
       </c>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>163</v>
       </c>
@@ -4359,17 +4471,20 @@
       <c r="C34">
         <v>947</v>
       </c>
-      <c r="E34" t="s">
+      <c r="D34" s="22">
+        <v>1827697</v>
+      </c>
+      <c r="F34" t="s">
         <v>164</v>
       </c>
-      <c r="F34">
+      <c r="G34">
         <v>5927047</v>
       </c>
-      <c r="G34">
+      <c r="H34">
         <v>5826820</v>
       </c>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>165</v>
       </c>
@@ -4379,17 +4494,20 @@
       <c r="C35">
         <v>1013</v>
       </c>
-      <c r="E35" t="s">
+      <c r="D35" s="22">
+        <v>1824127</v>
+      </c>
+      <c r="F35" t="s">
         <v>166</v>
       </c>
-      <c r="F35">
+      <c r="G35">
         <v>12.3</v>
       </c>
-      <c r="G35">
+      <c r="H35">
         <v>12.2</v>
       </c>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>167</v>
       </c>
@@ -4399,17 +4517,20 @@
       <c r="C36">
         <v>959</v>
       </c>
-      <c r="E36" t="s">
+      <c r="D36" s="22">
+        <v>1824127</v>
+      </c>
+      <c r="F36" t="s">
         <v>168</v>
       </c>
-      <c r="F36">
+      <c r="G36">
         <v>34.799999999999997</v>
       </c>
-      <c r="G36">
+      <c r="H36">
         <v>39.1</v>
       </c>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>169</v>
       </c>
@@ -4419,17 +4540,20 @@
       <c r="C37">
         <v>966</v>
       </c>
-      <c r="E37" t="s">
+      <c r="D37" s="22">
+        <v>1824127</v>
+      </c>
+      <c r="F37" t="s">
         <v>170</v>
       </c>
-      <c r="F37">
+      <c r="G37">
         <v>40.4</v>
       </c>
-      <c r="G37">
+      <c r="H37">
         <v>43.8</v>
       </c>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>171</v>
       </c>
@@ -4439,17 +4563,20 @@
       <c r="C38">
         <v>987</v>
       </c>
-      <c r="E38" t="s">
+      <c r="D38" s="22">
+        <v>1824127</v>
+      </c>
+      <c r="F38" t="s">
         <v>172</v>
       </c>
-      <c r="F38">
+      <c r="G38">
         <v>0.49</v>
       </c>
-      <c r="G38">
+      <c r="H38">
         <v>0.39</v>
       </c>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>173</v>
       </c>
@@ -4459,17 +4586,20 @@
       <c r="C39">
         <v>967</v>
       </c>
-      <c r="E39" t="s">
+      <c r="D39" s="22">
+        <v>1824127</v>
+      </c>
+      <c r="F39" t="s">
         <v>174</v>
       </c>
-      <c r="F39">
+      <c r="G39">
         <v>4.88</v>
       </c>
-      <c r="G39">
+      <c r="H39">
         <v>4.16</v>
       </c>
     </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>175</v>
       </c>
@@ -4479,17 +4609,20 @@
       <c r="C40">
         <v>927</v>
       </c>
-      <c r="E40" t="s">
+      <c r="D40" s="22">
+        <v>1824127</v>
+      </c>
+      <c r="F40" t="s">
         <v>176</v>
       </c>
-      <c r="F40">
+      <c r="G40">
         <v>4.88</v>
       </c>
-      <c r="G40">
+      <c r="H40">
         <v>4.16</v>
       </c>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>177</v>
       </c>
@@ -4499,17 +4632,20 @@
       <c r="C41">
         <v>969</v>
       </c>
-      <c r="E41" t="s">
+      <c r="D41" s="22">
+        <v>1824127</v>
+      </c>
+      <c r="F41" t="s">
         <v>178</v>
-      </c>
-      <c r="F41">
-        <v>0.16</v>
       </c>
       <c r="G41">
         <v>0.16</v>
       </c>
-    </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H41">
+        <v>0.16</v>
+      </c>
+    </row>
+    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>179</v>
       </c>
@@ -4519,17 +4655,20 @@
       <c r="C42">
         <v>940</v>
       </c>
-      <c r="E42" t="s">
+      <c r="D42" s="22">
+        <v>1824127</v>
+      </c>
+      <c r="F42" t="s">
         <v>180</v>
       </c>
-      <c r="F42">
+      <c r="G42">
         <v>1.61</v>
       </c>
-      <c r="G42">
+      <c r="H42">
         <v>1.68</v>
       </c>
     </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>181</v>
       </c>
@@ -4539,17 +4678,20 @@
       <c r="C43">
         <v>1056</v>
       </c>
-      <c r="E43" t="s">
+      <c r="D43" s="22">
+        <v>1824126</v>
+      </c>
+      <c r="F43" t="s">
         <v>182</v>
       </c>
-      <c r="F43">
+      <c r="G43">
         <v>1.61</v>
       </c>
-      <c r="G43">
+      <c r="H43">
         <v>1.68</v>
       </c>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>183</v>
       </c>
@@ -4559,17 +4701,20 @@
       <c r="C44">
         <v>1016</v>
       </c>
-      <c r="E44" t="s">
+      <c r="D44" s="22">
+        <v>1824126</v>
+      </c>
+      <c r="F44" t="s">
         <v>184</v>
       </c>
-      <c r="F44">
+      <c r="G44">
         <v>3</v>
       </c>
-      <c r="G44">
+      <c r="H44">
         <v>2.5</v>
       </c>
     </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>185</v>
       </c>
@@ -4579,17 +4724,20 @@
       <c r="C45">
         <v>910</v>
       </c>
-      <c r="E45" t="s">
+      <c r="D45" s="22">
+        <v>1824126</v>
+      </c>
+      <c r="F45" t="s">
         <v>186</v>
       </c>
-      <c r="F45">
+      <c r="G45">
         <v>11.18</v>
       </c>
-      <c r="G45">
+      <c r="H45">
         <v>11.57</v>
       </c>
     </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>187</v>
       </c>
@@ -4599,17 +4747,20 @@
       <c r="C46">
         <v>883</v>
       </c>
-      <c r="E46" t="s">
+      <c r="D46" s="22">
+        <v>1824126</v>
+      </c>
+      <c r="F46" t="s">
         <v>188</v>
       </c>
-      <c r="F46">
+      <c r="G46">
         <v>11.18</v>
       </c>
-      <c r="G46">
+      <c r="H46">
         <v>11.57</v>
       </c>
     </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>189</v>
       </c>
@@ -4619,17 +4770,20 @@
       <c r="C47">
         <v>943</v>
       </c>
-      <c r="E47" t="s">
+      <c r="D47" s="22">
+        <v>90</v>
+      </c>
+      <c r="F47" t="s">
         <v>190</v>
       </c>
-      <c r="F47">
+      <c r="G47">
         <v>3483019</v>
       </c>
-      <c r="G47">
+      <c r="H47">
         <v>3576470</v>
       </c>
     </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>191</v>
       </c>
@@ -4639,17 +4793,20 @@
       <c r="C48">
         <v>918</v>
       </c>
-      <c r="E48" t="s">
+      <c r="D48" s="22">
+        <v>1820564</v>
+      </c>
+      <c r="F48" t="s">
         <v>192</v>
-      </c>
-      <c r="F48">
-        <v>100</v>
       </c>
       <c r="G48">
         <v>100</v>
       </c>
-    </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H48">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="49" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>193</v>
       </c>
@@ -4659,17 +4816,20 @@
       <c r="C49">
         <v>900</v>
       </c>
-      <c r="E49" t="s">
+      <c r="D49" s="22">
+        <v>1820564</v>
+      </c>
+      <c r="F49" t="s">
         <v>194</v>
       </c>
-      <c r="F49">
+      <c r="G49">
         <v>1213634</v>
       </c>
-      <c r="G49">
+      <c r="H49">
         <v>1399966</v>
       </c>
     </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>195</v>
       </c>
@@ -4679,17 +4839,20 @@
       <c r="C50">
         <v>886</v>
       </c>
-      <c r="E50" t="s">
+      <c r="D50" s="22">
+        <v>1820564</v>
+      </c>
+      <c r="F50" t="s">
         <v>196</v>
       </c>
-      <c r="F50">
+      <c r="G50">
         <v>40.4</v>
       </c>
-      <c r="G50">
+      <c r="H50">
         <v>43.8</v>
       </c>
     </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>197</v>
       </c>
@@ -4699,17 +4862,20 @@
       <c r="C51">
         <v>920</v>
       </c>
-      <c r="E51" t="s">
+      <c r="D51" s="22">
+        <v>1820563</v>
+      </c>
+      <c r="F51" t="s">
         <v>198</v>
       </c>
-      <c r="F51">
+      <c r="G51">
         <v>4704</v>
       </c>
-      <c r="G51">
+      <c r="H51">
         <v>3728</v>
       </c>
     </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>199</v>
       </c>
@@ -4719,17 +4885,20 @@
       <c r="C52">
         <v>965</v>
       </c>
-      <c r="E52" t="s">
+      <c r="D52" s="22">
+        <v>1820563</v>
+      </c>
+      <c r="F52" t="s">
         <v>200</v>
       </c>
-      <c r="F52">
+      <c r="G52">
         <v>1132</v>
       </c>
-      <c r="G52">
+      <c r="H52">
         <v>1211</v>
       </c>
     </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>201</v>
       </c>
@@ -4739,8 +4908,11 @@
       <c r="C53">
         <v>1023</v>
       </c>
-    </row>
-    <row r="54" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="D53" s="22">
+        <v>1820563</v>
+      </c>
+    </row>
+    <row r="54" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>202</v>
       </c>
@@ -4750,11 +4922,14 @@
       <c r="C54">
         <v>1001</v>
       </c>
-      <c r="E54" t="s">
+      <c r="D54" s="22">
+        <v>1820563</v>
+      </c>
+      <c r="F54" t="s">
         <v>203</v>
       </c>
     </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>204</v>
       </c>
@@ -4764,17 +4939,20 @@
       <c r="C55">
         <v>1012</v>
       </c>
-      <c r="E55" t="s">
+      <c r="D55" s="22">
+        <v>90</v>
+      </c>
+      <c r="F55" t="s">
         <v>154</v>
       </c>
-      <c r="F55">
+      <c r="G55">
         <v>2842228</v>
       </c>
-      <c r="G55">
+      <c r="H55">
         <v>2776101</v>
       </c>
     </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>205</v>
       </c>
@@ -4784,17 +4962,20 @@
       <c r="C56">
         <v>975</v>
       </c>
-      <c r="E56" t="s">
+      <c r="D56" s="22">
+        <v>1820563</v>
+      </c>
+      <c r="F56" t="s">
         <v>156</v>
       </c>
-      <c r="F56">
+      <c r="G56">
         <v>26</v>
       </c>
-      <c r="G56">
+      <c r="H56">
         <v>25.4</v>
       </c>
     </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>206</v>
       </c>
@@ -4804,17 +4985,20 @@
       <c r="C57">
         <v>1006</v>
       </c>
-      <c r="E57" t="s">
+      <c r="D57" s="22">
+        <v>1820563</v>
+      </c>
+      <c r="F57" t="s">
         <v>158</v>
       </c>
-      <c r="F57">
+      <c r="G57">
         <v>2842</v>
       </c>
-      <c r="G57">
+      <c r="H57">
         <v>2776</v>
       </c>
     </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>207</v>
       </c>
@@ -4824,42 +5008,54 @@
       <c r="C58">
         <v>999</v>
       </c>
-      <c r="E58" t="s">
+      <c r="D58" s="22">
+        <v>1820563</v>
+      </c>
+      <c r="F58" t="s">
         <v>160</v>
       </c>
-      <c r="F58">
+      <c r="G58">
         <v>15197020</v>
       </c>
-      <c r="G58">
+      <c r="H58">
         <v>14607810</v>
       </c>
     </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="E59" t="s">
+    <row r="59" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="F59" t="s">
         <v>162</v>
       </c>
-      <c r="F59">
+      <c r="G59">
         <v>31.5</v>
       </c>
-      <c r="G59">
+      <c r="H59">
         <v>30.6</v>
       </c>
     </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>152</v>
       </c>
-      <c r="E60" t="s">
+      <c r="B60" t="s">
+        <v>68</v>
+      </c>
+      <c r="C60" t="s">
+        <v>84</v>
+      </c>
+      <c r="D60" t="s">
+        <v>282</v>
+      </c>
+      <c r="F60" t="s">
         <v>164</v>
       </c>
-      <c r="F60">
+      <c r="G60">
         <v>15197020</v>
       </c>
-      <c r="G60">
+      <c r="H60">
         <v>14607810</v>
       </c>
     </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>208</v>
       </c>
@@ -4869,17 +5065,20 @@
       <c r="C61">
         <v>274</v>
       </c>
-      <c r="E61" t="s">
+      <c r="D61" s="22">
+        <v>1831275</v>
+      </c>
+      <c r="F61" t="s">
         <v>166</v>
       </c>
-      <c r="F61">
+      <c r="G61">
         <v>31.5</v>
       </c>
-      <c r="G61">
+      <c r="H61">
         <v>30.6</v>
       </c>
     </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>209</v>
       </c>
@@ -4889,17 +5088,20 @@
       <c r="C62">
         <v>274</v>
       </c>
-      <c r="E62" t="s">
+      <c r="D62" s="22">
+        <v>1831275</v>
+      </c>
+      <c r="F62" t="s">
         <v>168</v>
       </c>
-      <c r="F62">
+      <c r="G62">
         <v>54.6</v>
       </c>
-      <c r="G62">
+      <c r="H62">
         <v>58.4</v>
       </c>
     </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>210</v>
       </c>
@@ -4909,17 +5111,20 @@
       <c r="C63">
         <v>302</v>
       </c>
-      <c r="E63" t="s">
+      <c r="D63" s="22">
+        <v>1831275</v>
+      </c>
+      <c r="F63" t="s">
         <v>170</v>
       </c>
-      <c r="F63">
+      <c r="G63">
         <v>63.3</v>
       </c>
-      <c r="G63">
+      <c r="H63">
         <v>65.400000000000006</v>
       </c>
     </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>211</v>
       </c>
@@ -4929,17 +5134,20 @@
       <c r="C64">
         <v>305</v>
       </c>
-      <c r="E64" t="s">
+      <c r="D64" s="22">
+        <v>1831275</v>
+      </c>
+      <c r="F64" t="s">
         <v>172</v>
       </c>
-      <c r="F64">
+      <c r="G64">
         <v>1.49</v>
       </c>
-      <c r="G64">
+      <c r="H64">
         <v>1.33</v>
       </c>
     </row>
-    <row r="65" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>212</v>
       </c>
@@ -4949,17 +5157,20 @@
       <c r="C65">
         <v>300</v>
       </c>
-      <c r="E65" t="s">
+      <c r="D65" s="22">
+        <v>1831275</v>
+      </c>
+      <c r="F65" t="s">
         <v>174</v>
       </c>
-      <c r="F65">
+      <c r="G65">
         <v>7.99</v>
       </c>
-      <c r="G65">
+      <c r="H65">
         <v>7</v>
       </c>
     </row>
-    <row r="66" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>213</v>
       </c>
@@ -4969,17 +5180,20 @@
       <c r="C66">
         <v>247</v>
       </c>
-      <c r="E66" t="s">
+      <c r="D66" s="22">
+        <v>1831275</v>
+      </c>
+      <c r="F66" t="s">
         <v>176</v>
       </c>
-      <c r="F66">
+      <c r="G66">
         <v>7.99</v>
       </c>
-      <c r="G66">
+      <c r="H66">
         <v>7</v>
       </c>
     </row>
-    <row r="67" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>214</v>
       </c>
@@ -4989,17 +5203,20 @@
       <c r="C67">
         <v>256</v>
       </c>
-      <c r="E67" t="s">
+      <c r="D67" s="22">
+        <v>1831275</v>
+      </c>
+      <c r="F67" t="s">
         <v>178</v>
       </c>
-      <c r="F67">
+      <c r="G67">
         <v>0.42</v>
       </c>
-      <c r="G67">
+      <c r="H67">
         <v>0.43</v>
       </c>
     </row>
-    <row r="68" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>215</v>
       </c>
@@ -5009,17 +5226,20 @@
       <c r="C68">
         <v>242</v>
       </c>
-      <c r="E68" t="s">
+      <c r="D68" s="22">
+        <v>1831275</v>
+      </c>
+      <c r="F68" t="s">
         <v>180</v>
-      </c>
-      <c r="F68">
-        <v>2.25</v>
       </c>
       <c r="G68">
         <v>2.25</v>
       </c>
-    </row>
-    <row r="69" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H68">
+        <v>2.25</v>
+      </c>
+    </row>
+    <row r="69" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>216</v>
       </c>
@@ -5029,17 +5249,20 @@
       <c r="C69">
         <v>222</v>
       </c>
-      <c r="E69" t="s">
+      <c r="D69" s="22">
+        <v>1831275</v>
+      </c>
+      <c r="F69" t="s">
         <v>182</v>
-      </c>
-      <c r="F69">
-        <v>2.25</v>
       </c>
       <c r="G69">
         <v>2.25</v>
       </c>
-    </row>
-    <row r="70" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H69">
+        <v>2.25</v>
+      </c>
+    </row>
+    <row r="70" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>217</v>
       </c>
@@ -5049,17 +5272,20 @@
       <c r="C70">
         <v>249</v>
       </c>
-      <c r="E70" t="s">
+      <c r="D70" s="22">
+        <v>1831275</v>
+      </c>
+      <c r="F70" t="s">
         <v>184</v>
       </c>
-      <c r="F70">
+      <c r="G70">
         <v>3.6</v>
       </c>
-      <c r="G70">
+      <c r="H70">
         <v>3.1</v>
       </c>
     </row>
-    <row r="71" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>218</v>
       </c>
@@ -5069,17 +5295,20 @@
       <c r="C71">
         <v>207</v>
       </c>
-      <c r="E71" t="s">
+      <c r="D71" s="22">
+        <v>1831275</v>
+      </c>
+      <c r="F71" t="s">
         <v>186</v>
       </c>
-      <c r="F71">
+      <c r="G71">
         <v>5.79</v>
       </c>
-      <c r="G71">
+      <c r="H71">
         <v>5.78</v>
       </c>
     </row>
-    <row r="72" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>219</v>
       </c>
@@ -5089,17 +5318,20 @@
       <c r="C72">
         <v>207</v>
       </c>
-      <c r="E72" t="s">
+      <c r="D72" s="22">
+        <v>1831275</v>
+      </c>
+      <c r="F72" t="s">
         <v>188</v>
       </c>
-      <c r="F72">
+      <c r="G72">
         <v>5.79</v>
       </c>
-      <c r="G72">
+      <c r="H72">
         <v>5.78</v>
       </c>
     </row>
-    <row r="73" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>220</v>
       </c>
@@ -5109,17 +5341,20 @@
       <c r="C73">
         <v>199</v>
       </c>
-      <c r="E73" t="s">
+      <c r="D73" s="22">
+        <v>1831274</v>
+      </c>
+      <c r="F73" t="s">
         <v>190</v>
       </c>
-      <c r="F73">
+      <c r="G73">
         <v>3483019</v>
       </c>
-      <c r="G73">
+      <c r="H73">
         <v>3576470</v>
       </c>
     </row>
-    <row r="74" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>221</v>
       </c>
@@ -5129,17 +5364,20 @@
       <c r="C74">
         <v>205</v>
       </c>
-      <c r="E74" t="s">
+      <c r="D74" s="22">
+        <v>1831274</v>
+      </c>
+      <c r="F74" t="s">
         <v>192</v>
-      </c>
-      <c r="F74">
-        <v>100</v>
       </c>
       <c r="G74">
         <v>100</v>
       </c>
-    </row>
-    <row r="75" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H74">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="75" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>222</v>
       </c>
@@ -5149,17 +5387,20 @@
       <c r="C75">
         <v>214</v>
       </c>
-      <c r="E75" t="s">
+      <c r="D75" s="22">
+        <v>1831274</v>
+      </c>
+      <c r="F75" t="s">
         <v>194</v>
       </c>
-      <c r="F75">
+      <c r="G75">
         <v>1901603</v>
       </c>
-      <c r="G75">
+      <c r="H75">
         <v>2086918</v>
       </c>
     </row>
-    <row r="76" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>223</v>
       </c>
@@ -5169,17 +5410,20 @@
       <c r="C76">
         <v>216</v>
       </c>
-      <c r="E76" t="s">
+      <c r="D76" s="22">
+        <v>1831274</v>
+      </c>
+      <c r="F76" t="s">
         <v>196</v>
       </c>
-      <c r="F76">
+      <c r="G76">
         <v>63.3</v>
       </c>
-      <c r="G76">
+      <c r="H76">
         <v>65.400000000000006</v>
       </c>
     </row>
-    <row r="77" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>224</v>
       </c>
@@ -5189,17 +5433,20 @@
       <c r="C77">
         <v>220</v>
       </c>
-      <c r="E77" t="s">
+      <c r="D77" s="22">
+        <v>1831274</v>
+      </c>
+      <c r="F77" t="s">
         <v>198</v>
       </c>
-      <c r="F77">
+      <c r="G77">
         <v>4704</v>
       </c>
-      <c r="G77">
+      <c r="H77">
         <v>3728</v>
       </c>
     </row>
-    <row r="78" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>225</v>
       </c>
@@ -5209,17 +5456,20 @@
       <c r="C78">
         <v>191</v>
       </c>
-      <c r="E78" t="s">
+      <c r="D78" s="22">
+        <v>1831274</v>
+      </c>
+      <c r="F78" t="s">
         <v>200</v>
       </c>
-      <c r="F78">
+      <c r="G78">
         <v>1821</v>
       </c>
-      <c r="G78">
+      <c r="H78">
         <v>1845</v>
       </c>
     </row>
-    <row r="79" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
         <v>226</v>
       </c>
@@ -5229,8 +5479,11 @@
       <c r="C79">
         <v>194</v>
       </c>
-    </row>
-    <row r="80" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="D79" s="22">
+        <v>1831274</v>
+      </c>
+    </row>
+    <row r="80" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>227</v>
       </c>
@@ -5240,8 +5493,11 @@
       <c r="C80">
         <v>173</v>
       </c>
-    </row>
-    <row r="81" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D80" s="22">
+        <v>1831274</v>
+      </c>
+    </row>
+    <row r="81" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>228</v>
       </c>
@@ -5251,8 +5507,11 @@
       <c r="C81">
         <v>173</v>
       </c>
-    </row>
-    <row r="82" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D81" s="22">
+        <v>1827697</v>
+      </c>
+    </row>
+    <row r="82" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
         <v>229</v>
       </c>
@@ -5262,8 +5521,11 @@
       <c r="C82">
         <v>190</v>
       </c>
-    </row>
-    <row r="83" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D82" s="22">
+        <v>1827697</v>
+      </c>
+    </row>
+    <row r="83" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
         <v>230</v>
       </c>
@@ -5273,8 +5535,11 @@
       <c r="C83">
         <v>179</v>
       </c>
-    </row>
-    <row r="84" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D83" s="22">
+        <v>1827697</v>
+      </c>
+    </row>
+    <row r="84" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
         <v>231</v>
       </c>
@@ -5284,8 +5549,11 @@
       <c r="C84">
         <v>168</v>
       </c>
-    </row>
-    <row r="85" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D84" s="22">
+        <v>1827697</v>
+      </c>
+    </row>
+    <row r="85" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
         <v>232</v>
       </c>
@@ -5295,8 +5563,11 @@
       <c r="C85">
         <v>151</v>
       </c>
-    </row>
-    <row r="86" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D85" s="22">
+        <v>1827697</v>
+      </c>
+    </row>
+    <row r="86" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
         <v>233</v>
       </c>
@@ -5306,8 +5577,11 @@
       <c r="C86">
         <v>150</v>
       </c>
-    </row>
-    <row r="87" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D86" s="22">
+        <v>1827697</v>
+      </c>
+    </row>
+    <row r="87" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
         <v>234</v>
       </c>
@@ -5317,8 +5591,11 @@
       <c r="C87">
         <v>140</v>
       </c>
-    </row>
-    <row r="88" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D87" s="22">
+        <v>1827697</v>
+      </c>
+    </row>
+    <row r="88" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
         <v>235</v>
       </c>
@@ -5328,8 +5605,11 @@
       <c r="C88">
         <v>142</v>
       </c>
-    </row>
-    <row r="89" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D88" s="22">
+        <v>1827697</v>
+      </c>
+    </row>
+    <row r="89" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
         <v>236</v>
       </c>
@@ -5339,8 +5619,11 @@
       <c r="C89">
         <v>148</v>
       </c>
-    </row>
-    <row r="90" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D89" s="22">
+        <v>1827697</v>
+      </c>
+    </row>
+    <row r="90" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
         <v>237</v>
       </c>
@@ -5350,8 +5633,11 @@
       <c r="C90">
         <v>133</v>
       </c>
-    </row>
-    <row r="91" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D90" s="22">
+        <v>1827697</v>
+      </c>
+    </row>
+    <row r="91" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
         <v>238</v>
       </c>
@@ -5361,8 +5647,11 @@
       <c r="C91">
         <v>218</v>
       </c>
-    </row>
-    <row r="92" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D91" s="22">
+        <v>1827697</v>
+      </c>
+    </row>
+    <row r="92" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
         <v>239</v>
       </c>
@@ -5372,8 +5661,11 @@
       <c r="C92">
         <v>210</v>
       </c>
-    </row>
-    <row r="93" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D92" s="22">
+        <v>1827697</v>
+      </c>
+    </row>
+    <row r="93" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
         <v>240</v>
       </c>
@@ -5383,8 +5675,11 @@
       <c r="C93">
         <v>220</v>
       </c>
-    </row>
-    <row r="94" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D93" s="22">
+        <v>1824127</v>
+      </c>
+    </row>
+    <row r="94" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
         <v>241</v>
       </c>
@@ -5394,8 +5689,11 @@
       <c r="C94">
         <v>196</v>
       </c>
-    </row>
-    <row r="95" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D94" s="22">
+        <v>1824127</v>
+      </c>
+    </row>
+    <row r="95" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
         <v>242</v>
       </c>
@@ -5405,8 +5703,11 @@
       <c r="C95">
         <v>174</v>
       </c>
-    </row>
-    <row r="96" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D95" s="22">
+        <v>1824127</v>
+      </c>
+    </row>
+    <row r="96" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
         <v>243</v>
       </c>
@@ -5416,8 +5717,11 @@
       <c r="C96">
         <v>192</v>
       </c>
-    </row>
-    <row r="97" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D96" s="22">
+        <v>1824127</v>
+      </c>
+    </row>
+    <row r="97" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
         <v>244</v>
       </c>
@@ -5427,8 +5731,11 @@
       <c r="C97">
         <v>171</v>
       </c>
-    </row>
-    <row r="98" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D97" s="22">
+        <v>1824127</v>
+      </c>
+    </row>
+    <row r="98" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
         <v>245</v>
       </c>
@@ -5438,8 +5745,11 @@
       <c r="C98">
         <v>168</v>
       </c>
-    </row>
-    <row r="99" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D98" s="22">
+        <v>1824127</v>
+      </c>
+    </row>
+    <row r="99" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
         <v>246</v>
       </c>
@@ -5449,8 +5759,11 @@
       <c r="C99">
         <v>202</v>
       </c>
-    </row>
-    <row r="100" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D99" s="22">
+        <v>1824127</v>
+      </c>
+    </row>
+    <row r="100" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
         <v>247</v>
       </c>
@@ -5460,8 +5773,11 @@
       <c r="C100">
         <v>174</v>
       </c>
-    </row>
-    <row r="101" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D100" s="22">
+        <v>1824127</v>
+      </c>
+    </row>
+    <row r="101" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
         <v>248</v>
       </c>
@@ -5471,8 +5787,11 @@
       <c r="C101">
         <v>212</v>
       </c>
-    </row>
-    <row r="102" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D101" s="22">
+        <v>1824126</v>
+      </c>
+    </row>
+    <row r="102" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
         <v>249</v>
       </c>
@@ -5482,8 +5801,11 @@
       <c r="C102">
         <v>221</v>
       </c>
-    </row>
-    <row r="103" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D102" s="22">
+        <v>1824126</v>
+      </c>
+    </row>
+    <row r="103" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
         <v>250</v>
       </c>
@@ -5493,8 +5815,11 @@
       <c r="C103">
         <v>172</v>
       </c>
-    </row>
-    <row r="104" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D103" s="22">
+        <v>1824126</v>
+      </c>
+    </row>
+    <row r="104" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
         <v>251</v>
       </c>
@@ -5504,8 +5829,11 @@
       <c r="C104">
         <v>179</v>
       </c>
-    </row>
-    <row r="105" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D104" s="22">
+        <v>1824126</v>
+      </c>
+    </row>
+    <row r="105" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
         <v>252</v>
       </c>
@@ -5515,8 +5843,11 @@
       <c r="C105">
         <v>205</v>
       </c>
-    </row>
-    <row r="106" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D105" s="22">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="106" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
         <v>253</v>
       </c>
@@ -5526,8 +5857,11 @@
       <c r="C106">
         <v>197</v>
       </c>
-    </row>
-    <row r="107" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D106" s="22">
+        <v>1820564</v>
+      </c>
+    </row>
+    <row r="107" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
         <v>254</v>
       </c>
@@ -5537,8 +5871,11 @@
       <c r="C107">
         <v>179</v>
       </c>
-    </row>
-    <row r="108" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D107" s="22">
+        <v>1820564</v>
+      </c>
+    </row>
+    <row r="108" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
         <v>255</v>
       </c>
@@ -5548,8 +5885,11 @@
       <c r="C108">
         <v>182</v>
       </c>
-    </row>
-    <row r="109" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D108" s="22">
+        <v>1820564</v>
+      </c>
+    </row>
+    <row r="109" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
         <v>256</v>
       </c>
@@ -5559,8 +5899,11 @@
       <c r="C109">
         <v>154</v>
       </c>
-    </row>
-    <row r="110" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D109" s="22">
+        <v>1820563</v>
+      </c>
+    </row>
+    <row r="110" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
         <v>257</v>
       </c>
@@ -5570,8 +5913,11 @@
       <c r="C110">
         <v>219</v>
       </c>
-    </row>
-    <row r="111" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D110" s="22">
+        <v>1820563</v>
+      </c>
+    </row>
+    <row r="111" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
         <v>258</v>
       </c>
@@ -5581,8 +5927,11 @@
       <c r="C111">
         <v>203</v>
       </c>
-    </row>
-    <row r="112" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D111" s="22">
+        <v>1820563</v>
+      </c>
+    </row>
+    <row r="112" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
         <v>259</v>
       </c>
@@ -5592,8 +5941,11 @@
       <c r="C112">
         <v>208</v>
       </c>
-    </row>
-    <row r="113" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D112" s="22">
+        <v>1820563</v>
+      </c>
+    </row>
+    <row r="113" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
         <v>260</v>
       </c>
@@ -5603,8 +5955,11 @@
       <c r="C113">
         <v>211</v>
       </c>
-    </row>
-    <row r="114" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D113" s="22">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="114" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
         <v>261</v>
       </c>
@@ -5614,8 +5969,11 @@
       <c r="C114">
         <v>186</v>
       </c>
-    </row>
-    <row r="115" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D114" s="22">
+        <v>1820563</v>
+      </c>
+    </row>
+    <row r="115" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
         <v>262</v>
       </c>
@@ -5625,8 +5983,11 @@
       <c r="C115">
         <v>190</v>
       </c>
-    </row>
-    <row r="116" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D115" s="22">
+        <v>1820563</v>
+      </c>
+    </row>
+    <row r="116" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
         <v>263</v>
       </c>
@@ -5636,13 +5997,25 @@
       <c r="C116">
         <v>200</v>
       </c>
-    </row>
-    <row r="118" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D116" s="22">
+        <v>1820563</v>
+      </c>
+    </row>
+    <row r="118" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
         <v>203</v>
       </c>
-    </row>
-    <row r="119" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B118" t="s">
+        <v>68</v>
+      </c>
+      <c r="C118" t="s">
+        <v>84</v>
+      </c>
+      <c r="D118" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="119" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
         <v>208</v>
       </c>
@@ -5652,8 +6025,11 @@
       <c r="C119">
         <v>244</v>
       </c>
-    </row>
-    <row r="120" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D119" s="22">
+        <v>1831275</v>
+      </c>
+    </row>
+    <row r="120" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
         <v>209</v>
       </c>
@@ -5663,8 +6039,11 @@
       <c r="C120">
         <v>236</v>
       </c>
-    </row>
-    <row r="121" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D120" s="22">
+        <v>1831275</v>
+      </c>
+    </row>
+    <row r="121" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
         <v>210</v>
       </c>
@@ -5674,8 +6053,11 @@
       <c r="C121">
         <v>279</v>
       </c>
-    </row>
-    <row r="122" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D121" s="22">
+        <v>1831275</v>
+      </c>
+    </row>
+    <row r="122" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
         <v>211</v>
       </c>
@@ -5685,8 +6067,11 @@
       <c r="C122">
         <v>265</v>
       </c>
-    </row>
-    <row r="123" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D122" s="22">
+        <v>1831275</v>
+      </c>
+    </row>
+    <row r="123" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
         <v>212</v>
       </c>
@@ -5696,8 +6081,11 @@
       <c r="C123">
         <v>278</v>
       </c>
-    </row>
-    <row r="124" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D123" s="22">
+        <v>1831275</v>
+      </c>
+    </row>
+    <row r="124" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
         <v>213</v>
       </c>
@@ -5707,8 +6095,11 @@
       <c r="C124">
         <v>243</v>
       </c>
-    </row>
-    <row r="125" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D124" s="22">
+        <v>1831275</v>
+      </c>
+    </row>
+    <row r="125" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A125" t="s">
         <v>214</v>
       </c>
@@ -5718,8 +6109,11 @@
       <c r="C125">
         <v>230</v>
       </c>
-    </row>
-    <row r="126" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D125" s="22">
+        <v>1831275</v>
+      </c>
+    </row>
+    <row r="126" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A126" t="s">
         <v>215</v>
       </c>
@@ -5729,8 +6123,11 @@
       <c r="C126">
         <v>243</v>
       </c>
-    </row>
-    <row r="127" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D126" s="22">
+        <v>1831275</v>
+      </c>
+    </row>
+    <row r="127" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A127" t="s">
         <v>216</v>
       </c>
@@ -5740,8 +6137,11 @@
       <c r="C127">
         <v>218</v>
       </c>
-    </row>
-    <row r="128" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D127" s="22">
+        <v>1831275</v>
+      </c>
+    </row>
+    <row r="128" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A128" t="s">
         <v>217</v>
       </c>
@@ -5751,8 +6151,11 @@
       <c r="C128">
         <v>257</v>
       </c>
-    </row>
-    <row r="129" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D128" s="22">
+        <v>1831275</v>
+      </c>
+    </row>
+    <row r="129" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A129" t="s">
         <v>218</v>
       </c>
@@ -5762,8 +6165,11 @@
       <c r="C129">
         <v>228</v>
       </c>
-    </row>
-    <row r="130" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D129" s="22">
+        <v>1831275</v>
+      </c>
+    </row>
+    <row r="130" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A130" t="s">
         <v>219</v>
       </c>
@@ -5773,8 +6179,11 @@
       <c r="C130">
         <v>237</v>
       </c>
-    </row>
-    <row r="131" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D130" s="22">
+        <v>1831275</v>
+      </c>
+    </row>
+    <row r="131" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A131" t="s">
         <v>220</v>
       </c>
@@ -5784,8 +6193,11 @@
       <c r="C131">
         <v>214</v>
       </c>
-    </row>
-    <row r="132" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D131" s="22">
+        <v>1831274</v>
+      </c>
+    </row>
+    <row r="132" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A132" t="s">
         <v>221</v>
       </c>
@@ -5795,8 +6207,11 @@
       <c r="C132">
         <v>227</v>
       </c>
-    </row>
-    <row r="133" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D132" s="22">
+        <v>1831274</v>
+      </c>
+    </row>
+    <row r="133" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A133" t="s">
         <v>222</v>
       </c>
@@ -5806,8 +6221,11 @@
       <c r="C133">
         <v>271</v>
       </c>
-    </row>
-    <row r="134" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D133" s="22">
+        <v>1831274</v>
+      </c>
+    </row>
+    <row r="134" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A134" t="s">
         <v>223</v>
       </c>
@@ -5817,8 +6235,11 @@
       <c r="C134">
         <v>235</v>
       </c>
-    </row>
-    <row r="135" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D134" s="22">
+        <v>1831274</v>
+      </c>
+    </row>
+    <row r="135" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A135" t="s">
         <v>224</v>
       </c>
@@ -5828,8 +6249,11 @@
       <c r="C135">
         <v>232</v>
       </c>
-    </row>
-    <row r="136" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D135" s="22">
+        <v>1831274</v>
+      </c>
+    </row>
+    <row r="136" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A136" t="s">
         <v>225</v>
       </c>
@@ -5839,8 +6263,11 @@
       <c r="C136">
         <v>248</v>
       </c>
-    </row>
-    <row r="137" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D136" s="22">
+        <v>1831274</v>
+      </c>
+    </row>
+    <row r="137" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A137" t="s">
         <v>226</v>
       </c>
@@ -5850,8 +6277,11 @@
       <c r="C137">
         <v>262</v>
       </c>
-    </row>
-    <row r="138" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D137" s="22">
+        <v>1831274</v>
+      </c>
+    </row>
+    <row r="138" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A138" t="s">
         <v>227</v>
       </c>
@@ -5861,8 +6291,11 @@
       <c r="C138">
         <v>271</v>
       </c>
-    </row>
-    <row r="139" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D138" s="22">
+        <v>1831274</v>
+      </c>
+    </row>
+    <row r="139" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A139" t="s">
         <v>228</v>
       </c>
@@ -5872,8 +6305,11 @@
       <c r="C139">
         <v>230</v>
       </c>
-    </row>
-    <row r="140" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D139" s="22">
+        <v>1827697</v>
+      </c>
+    </row>
+    <row r="140" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A140" t="s">
         <v>229</v>
       </c>
@@ -5883,8 +6319,11 @@
       <c r="C140">
         <v>249</v>
       </c>
-    </row>
-    <row r="141" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D140" s="22">
+        <v>1827697</v>
+      </c>
+    </row>
+    <row r="141" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A141" t="s">
         <v>230</v>
       </c>
@@ -5894,8 +6333,11 @@
       <c r="C141">
         <v>236</v>
       </c>
-    </row>
-    <row r="142" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D141" s="22">
+        <v>1827697</v>
+      </c>
+    </row>
+    <row r="142" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A142" t="s">
         <v>231</v>
       </c>
@@ -5905,8 +6347,11 @@
       <c r="C142">
         <v>235</v>
       </c>
-    </row>
-    <row r="143" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D142" s="22">
+        <v>1827697</v>
+      </c>
+    </row>
+    <row r="143" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A143" t="s">
         <v>232</v>
       </c>
@@ -5916,8 +6361,11 @@
       <c r="C143">
         <v>217</v>
       </c>
-    </row>
-    <row r="144" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D143" s="22">
+        <v>1827697</v>
+      </c>
+    </row>
+    <row r="144" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A144" t="s">
         <v>233</v>
       </c>
@@ -5927,8 +6375,11 @@
       <c r="C144">
         <v>241</v>
       </c>
-    </row>
-    <row r="145" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D144" s="22">
+        <v>1827697</v>
+      </c>
+    </row>
+    <row r="145" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A145" t="s">
         <v>234</v>
       </c>
@@ -5938,8 +6389,11 @@
       <c r="C145">
         <v>259</v>
       </c>
-    </row>
-    <row r="146" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D145" s="22">
+        <v>1827697</v>
+      </c>
+    </row>
+    <row r="146" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A146" t="s">
         <v>235</v>
       </c>
@@ -5949,8 +6403,11 @@
       <c r="C146">
         <v>259</v>
       </c>
-    </row>
-    <row r="147" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D146" s="22">
+        <v>1827697</v>
+      </c>
+    </row>
+    <row r="147" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A147" t="s">
         <v>236</v>
       </c>
@@ -5960,8 +6417,11 @@
       <c r="C147">
         <v>256</v>
       </c>
-    </row>
-    <row r="148" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D147" s="22">
+        <v>1827697</v>
+      </c>
+    </row>
+    <row r="148" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A148" t="s">
         <v>237</v>
       </c>
@@ -5971,8 +6431,11 @@
       <c r="C148">
         <v>275</v>
       </c>
-    </row>
-    <row r="149" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D148" s="22">
+        <v>1827697</v>
+      </c>
+    </row>
+    <row r="149" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A149" t="s">
         <v>238</v>
       </c>
@@ -5982,8 +6445,11 @@
       <c r="C149">
         <v>308</v>
       </c>
-    </row>
-    <row r="150" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D149" s="22">
+        <v>1827697</v>
+      </c>
+    </row>
+    <row r="150" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A150" t="s">
         <v>239</v>
       </c>
@@ -5993,8 +6459,11 @@
       <c r="C150">
         <v>331</v>
       </c>
-    </row>
-    <row r="151" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D150" s="22">
+        <v>1827697</v>
+      </c>
+    </row>
+    <row r="151" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A151" t="s">
         <v>240</v>
       </c>
@@ -6004,8 +6473,11 @@
       <c r="C151">
         <v>367</v>
       </c>
-    </row>
-    <row r="152" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D151" s="22">
+        <v>1824127</v>
+      </c>
+    </row>
+    <row r="152" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A152" t="s">
         <v>241</v>
       </c>
@@ -6015,8 +6487,11 @@
       <c r="C152">
         <v>363</v>
       </c>
-    </row>
-    <row r="153" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D152" s="22">
+        <v>1824127</v>
+      </c>
+    </row>
+    <row r="153" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A153" t="s">
         <v>242</v>
       </c>
@@ -6026,8 +6501,11 @@
       <c r="C153">
         <v>358</v>
       </c>
-    </row>
-    <row r="154" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D153" s="22">
+        <v>1824127</v>
+      </c>
+    </row>
+    <row r="154" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A154" t="s">
         <v>243</v>
       </c>
@@ -6037,8 +6515,11 @@
       <c r="C154">
         <v>360</v>
       </c>
-    </row>
-    <row r="155" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D154" s="22">
+        <v>1824127</v>
+      </c>
+    </row>
+    <row r="155" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A155" t="s">
         <v>244</v>
       </c>
@@ -6048,8 +6529,11 @@
       <c r="C155">
         <v>366</v>
       </c>
-    </row>
-    <row r="156" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D155" s="22">
+        <v>1824127</v>
+      </c>
+    </row>
+    <row r="156" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A156" t="s">
         <v>245</v>
       </c>
@@ -6059,8 +6543,11 @@
       <c r="C156">
         <v>370</v>
       </c>
-    </row>
-    <row r="157" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D156" s="22">
+        <v>1824127</v>
+      </c>
+    </row>
+    <row r="157" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A157" t="s">
         <v>246</v>
       </c>
@@ -6070,8 +6557,11 @@
       <c r="C157">
         <v>385</v>
       </c>
-    </row>
-    <row r="158" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D157" s="22">
+        <v>1824127</v>
+      </c>
+    </row>
+    <row r="158" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A158" t="s">
         <v>247</v>
       </c>
@@ -6081,8 +6571,11 @@
       <c r="C158">
         <v>367</v>
       </c>
-    </row>
-    <row r="159" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D158" s="22">
+        <v>1824127</v>
+      </c>
+    </row>
+    <row r="159" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A159" t="s">
         <v>248</v>
       </c>
@@ -6092,8 +6585,11 @@
       <c r="C159">
         <v>433</v>
       </c>
-    </row>
-    <row r="160" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D159" s="22">
+        <v>1824126</v>
+      </c>
+    </row>
+    <row r="160" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A160" t="s">
         <v>249</v>
       </c>
@@ -6103,8 +6599,11 @@
       <c r="C160">
         <v>351</v>
       </c>
-    </row>
-    <row r="161" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D160" s="22">
+        <v>1824126</v>
+      </c>
+    </row>
+    <row r="161" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A161" t="s">
         <v>250</v>
       </c>
@@ -6114,8 +6613,11 @@
       <c r="C161">
         <v>338</v>
       </c>
-    </row>
-    <row r="162" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D161" s="22">
+        <v>1824126</v>
+      </c>
+    </row>
+    <row r="162" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A162" t="s">
         <v>251</v>
       </c>
@@ -6125,8 +6627,11 @@
       <c r="C162">
         <v>334</v>
       </c>
-    </row>
-    <row r="163" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D162" s="22">
+        <v>1824126</v>
+      </c>
+    </row>
+    <row r="163" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A163" t="s">
         <v>252</v>
       </c>
@@ -6136,8 +6641,11 @@
       <c r="C163">
         <v>341</v>
       </c>
-    </row>
-    <row r="164" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D163" s="22">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="164" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A164" t="s">
         <v>253</v>
       </c>
@@ -6147,8 +6655,11 @@
       <c r="C164">
         <v>342</v>
       </c>
-    </row>
-    <row r="165" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D164" s="22">
+        <v>1820564</v>
+      </c>
+    </row>
+    <row r="165" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A165" t="s">
         <v>254</v>
       </c>
@@ -6158,8 +6669,11 @@
       <c r="C165">
         <v>358</v>
       </c>
-    </row>
-    <row r="166" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D165" s="22">
+        <v>1820564</v>
+      </c>
+    </row>
+    <row r="166" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A166" t="s">
         <v>255</v>
       </c>
@@ -6169,8 +6683,11 @@
       <c r="C166">
         <v>328</v>
       </c>
-    </row>
-    <row r="167" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D166" s="22">
+        <v>1820564</v>
+      </c>
+    </row>
+    <row r="167" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A167" t="s">
         <v>256</v>
       </c>
@@ -6180,8 +6697,11 @@
       <c r="C167">
         <v>355</v>
       </c>
-    </row>
-    <row r="168" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D167" s="22">
+        <v>1820563</v>
+      </c>
+    </row>
+    <row r="168" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A168" t="s">
         <v>257</v>
       </c>
@@ -6191,8 +6711,11 @@
       <c r="C168">
         <v>340</v>
       </c>
-    </row>
-    <row r="169" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D168" s="22">
+        <v>1820563</v>
+      </c>
+    </row>
+    <row r="169" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A169" t="s">
         <v>258</v>
       </c>
@@ -6202,8 +6725,11 @@
       <c r="C169">
         <v>370</v>
       </c>
-    </row>
-    <row r="170" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D169" s="22">
+        <v>1820563</v>
+      </c>
+    </row>
+    <row r="170" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A170" t="s">
         <v>259</v>
       </c>
@@ -6213,8 +6739,11 @@
       <c r="C170">
         <v>333</v>
       </c>
-    </row>
-    <row r="171" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D170" s="22">
+        <v>1820563</v>
+      </c>
+    </row>
+    <row r="171" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A171" t="s">
         <v>260</v>
       </c>
@@ -6224,8 +6753,11 @@
       <c r="C171">
         <v>345</v>
       </c>
-    </row>
-    <row r="172" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D171" s="22">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="172" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A172" t="s">
         <v>261</v>
       </c>
@@ -6235,8 +6767,11 @@
       <c r="C172">
         <v>353</v>
       </c>
-    </row>
-    <row r="173" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D172" s="22">
+        <v>1820563</v>
+      </c>
+    </row>
+    <row r="173" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A173" t="s">
         <v>262</v>
       </c>
@@ -6246,8 +6781,11 @@
       <c r="C173">
         <v>365</v>
       </c>
-    </row>
-    <row r="174" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D173" s="22">
+        <v>1820563</v>
+      </c>
+    </row>
+    <row r="174" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A174" t="s">
         <v>263</v>
       </c>
@@ -6256,6 +6794,9 @@
       </c>
       <c r="C174">
         <v>350</v>
+      </c>
+      <c r="D174" s="22">
+        <v>1820563</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: agrega modo pp para penetración del árbol
Por qué:
- Algunos análisis necesitan leer la penetración como cambio absoluto en puntos porcentuales, no como variación relativa.

Qué cambió:
- Se permite nombrar hojas del segmento 2 con sufijo _pp para calcular penetración en puntos porcentuales.
- El generador de plantilla permite elegir entre variación porcentual y puntos porcentuales.
- Se actualiza la plantilla de entrada y la documentación del nuevo sufijo.

Impacto:
- El comportamiento actual se mantiene cuando no se selecciona nada o se usa %.
- Al usar _pp, solo cambia la tarjeta de % Penetracion; los colores y el resto del árbol se conservan.

Trade-offs o riesgos:
- Los nombres de hoja largos pueden recortarse por el límite de Excel, pero se preserva el sufijo operativo de unidad y modo.

Diferencia vs commit anterior:
- Este cambio se concentra en Segmento 2 y en el flujo de plantilla; el commit anterior ajustaba mapeos del Segmento 8.
</commit_message>
<xml_diff>
--- a/Plantilla_Entrada_5W1H.xlsx
+++ b/Plantilla_Entrada_5W1H.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\NavaG\Downloads\5W1H\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7588F95-FFB5-4E66-8D8F-55C8C4A5B660}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC6FB6C8-E3CA-4E1F-8C12-7C782D6E6FD4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="26010" windowHeight="20985" tabRatio="949" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="34605" windowHeight="20985" tabRatio="949" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="1" r:id="rId1"/>
@@ -1263,7 +1263,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="426" uniqueCount="292">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="429" uniqueCount="295">
   <si>
     <t>Plantilla de Entrada 5W1H</t>
   </si>
@@ -2139,13 +2139,22 @@
   </si>
   <si>
     <t>Liquido</t>
+  </si>
+  <si>
+    <t>Presentacion</t>
+  </si>
+  <si>
+    <t>% / pp</t>
+  </si>
+  <si>
+    <t>Muestra el valor de penetracion en variacion o en puntos porcentuales</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2200,8 +2209,16 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="12">
+  <fills count="13">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -2263,6 +2280,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="3" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -2285,7 +2308,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -2330,6 +2353,8 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2725,12 +2750,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C42"/>
+  <dimension ref="A1:F42"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="48" customWidth="1"/>
     <col min="2" max="2" width="32.140625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="13.42578125" customWidth="1"/>
+    <col min="4" max="4" width="12.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="21" x14ac:dyDescent="0.35">
@@ -2813,32 +2839,32 @@
         <v>9</v>
       </c>
     </row>
-    <row r="20" spans="1:3" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:6" ht="17.25" x14ac:dyDescent="0.3">
       <c r="A20" s="4" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" s="17" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" s="17" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" s="20" t="s">
         <v>43</v>
       </c>
@@ -2848,8 +2874,11 @@
       <c r="C26" s="20" t="s">
         <v>264</v>
       </c>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D26" s="20" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" s="23" t="s">
         <v>44</v>
       </c>
@@ -2857,8 +2886,8 @@
         <v>265</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A28" s="23" t="s">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A28" s="24" t="s">
         <v>279</v>
       </c>
       <c r="B28" t="s">
@@ -2867,16 +2896,23 @@
       <c r="C28" t="s">
         <v>276</v>
       </c>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D28" t="s">
+        <v>293</v>
+      </c>
+      <c r="F28" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" s="23" t="s">
         <v>45</v>
       </c>
       <c r="C29" t="s">
         <v>267</v>
       </c>
-    </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="F29" s="25"/>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" s="23" t="s">
         <v>46</v>
       </c>
@@ -2884,7 +2920,7 @@
         <v>272</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" s="23" t="s">
         <v>47</v>
       </c>
@@ -2892,7 +2928,7 @@
         <v>268</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" s="23" t="s">
         <v>284</v>
       </c>
@@ -2960,7 +2996,7 @@
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A40" s="23" t="s">
+      <c r="A40" s="24" t="s">
         <v>97</v>
       </c>
       <c r="C40" t="s">

</xml_diff>